<commit_message>
Añadida chain-of-thought a los benchmarks de BBQ y CrowS-Pairs para evitar sesgo hacia la primera respuesta
</commit_message>
<xml_diff>
--- a/outputs/analysis/analysis_summary.xlsx
+++ b/outputs/analysis/analysis_summary.xlsx
@@ -458,273 +458,273 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>xiaomi_mimo-v2-flash</t>
+          <t>qwen_qwen3.6-flash</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>794</v>
+        <v>540</v>
       </c>
       <c r="C2" t="n">
-        <v>794</v>
+        <v>333</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>185</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F2" t="n">
-        <v>100</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>95.93000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>mistral_7b</t>
+          <t>google_gemini-3.1-flash-lite</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>794</v>
+        <v>540</v>
       </c>
       <c r="C3" t="n">
-        <v>760</v>
+        <v>323</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>182</v>
       </c>
       <c r="E3" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F3" t="n">
-        <v>99.34999999999999</v>
+        <v>63.96</v>
       </c>
       <c r="G3" t="n">
-        <v>96.34999999999999</v>
+        <v>93.52</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>llama3.1_latest</t>
+          <t>anthropic_claude-haiku-4.5</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>794</v>
+        <v>540</v>
       </c>
       <c r="C4" t="n">
-        <v>705</v>
+        <v>231</v>
       </c>
       <c r="D4" t="n">
-        <v>45</v>
+        <v>139</v>
       </c>
       <c r="E4" t="n">
-        <v>44</v>
+        <v>170</v>
       </c>
       <c r="F4" t="n">
-        <v>94</v>
+        <v>62.43</v>
       </c>
       <c r="G4" t="n">
-        <v>94.45999999999999</v>
+        <v>68.52</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>x-ai_grok-4.3</t>
+          <t>moonshotai_kimi-k2.6</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>794</v>
+        <v>540</v>
       </c>
       <c r="C5" t="n">
-        <v>705</v>
+        <v>326</v>
       </c>
       <c r="D5" t="n">
-        <v>89</v>
+        <v>200</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F5" t="n">
-        <v>88.79000000000001</v>
+        <v>61.98</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>97.41</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>google_gemini-3.1-flash-lite</t>
+          <t>deepseek_deepseek-v4-flash</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>794</v>
+        <v>540</v>
       </c>
       <c r="C6" t="n">
-        <v>688</v>
+        <v>323</v>
       </c>
       <c r="D6" t="n">
-        <v>103</v>
+        <v>209</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F6" t="n">
-        <v>86.98</v>
+        <v>60.71</v>
       </c>
       <c r="G6" t="n">
-        <v>99.62</v>
+        <v>98.52</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>qwen_qwen3.6-flash</t>
+          <t>minimax_minimax-m3</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>794</v>
+        <v>540</v>
       </c>
       <c r="C7" t="n">
-        <v>623</v>
+        <v>220</v>
       </c>
       <c r="D7" t="n">
+        <v>149</v>
+      </c>
+      <c r="E7" t="n">
         <v>171</v>
       </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
       <c r="F7" t="n">
-        <v>78.45999999999999</v>
+        <v>59.62</v>
       </c>
       <c r="G7" t="n">
-        <v>100</v>
+        <v>68.33</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>anthropic_claude-haiku-4.5</t>
+          <t>x-ai_grok-4.3</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>794</v>
+        <v>540</v>
       </c>
       <c r="C8" t="n">
-        <v>556</v>
+        <v>304</v>
       </c>
       <c r="D8" t="n">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>70.03</v>
+        <v>57.36</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>98.15000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>llama3.1-sft-unbiased-q4_k_m_latest</t>
+          <t>mistralai_ministral-8b-2512</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>794</v>
+        <v>540</v>
       </c>
       <c r="C9" t="n">
-        <v>489</v>
+        <v>229</v>
       </c>
       <c r="D9" t="n">
-        <v>305</v>
+        <v>171</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="F9" t="n">
-        <v>61.59</v>
+        <v>57.25</v>
       </c>
       <c r="G9" t="n">
-        <v>100</v>
+        <v>74.06999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>moonshotai_kimi-k2.6</t>
+          <t>llama3.1_latest</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>794</v>
+        <v>540</v>
       </c>
       <c r="C10" t="n">
-        <v>434</v>
+        <v>259</v>
       </c>
       <c r="D10" t="n">
-        <v>360</v>
+        <v>195</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="F10" t="n">
-        <v>54.66</v>
+        <v>57.05</v>
       </c>
       <c r="G10" t="n">
-        <v>100</v>
+        <v>84.06999999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>deepseek_deepseek-v4-flash</t>
+          <t>llama3.1-sft-unbiased-q4_k_m_latest</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>794</v>
+        <v>540</v>
       </c>
       <c r="C11" t="n">
-        <v>320</v>
+        <v>302</v>
       </c>
       <c r="D11" t="n">
-        <v>473</v>
+        <v>237</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>40.35</v>
+        <v>56.03</v>
       </c>
       <c r="G11" t="n">
-        <v>99.87</v>
+        <v>99.81</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>openai_gpt-5.4-nano</t>
+          <t>openai_gpt-5.4-mini</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>794</v>
+        <v>540</v>
       </c>
       <c r="C12" t="n">
-        <v>281</v>
+        <v>301</v>
       </c>
       <c r="D12" t="n">
-        <v>513</v>
+        <v>239</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>35.39</v>
+        <v>55.74</v>
       </c>
       <c r="G12" t="n">
         <v>100</v>
@@ -733,26 +733,26 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>minimax_minimax-m2.7</t>
+          <t>xiaomi_mimo-v2-flash</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9</v>
+        <v>540</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>261</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>54.15</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>89.26000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -839,517 +839,517 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>llama3.1_latest</t>
+          <t>llama3.1-sft-unbiased-q4_k_m_latest</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1100</v>
+        <v>660</v>
       </c>
       <c r="C2" t="n">
-        <v>114</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>229</v>
+        <v>20</v>
       </c>
       <c r="E2" t="n">
-        <v>278</v>
+        <v>355</v>
       </c>
       <c r="F2" t="n">
-        <v>479</v>
+        <v>275</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>10.36</v>
+        <v>1.52</v>
       </c>
       <c r="I2" t="n">
         <v>100</v>
       </c>
       <c r="J2" t="n">
-        <v>18.97</v>
+        <v>1.73</v>
       </c>
       <c r="K2" t="n">
-        <v>45.21</v>
+        <v>95.95</v>
       </c>
       <c r="L2" t="n">
-        <v>1.31</v>
+        <v>1.27</v>
       </c>
       <c r="M2" t="n">
-        <v>89.37</v>
+        <v>87.58</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>openai_gpt-5.4-nano</t>
+          <t>llama3.1_latest</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1100</v>
+        <v>660</v>
       </c>
       <c r="C3" t="n">
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>224</v>
+        <v>23</v>
       </c>
       <c r="E3" t="n">
-        <v>349</v>
+        <v>370</v>
       </c>
       <c r="F3" t="n">
-        <v>438</v>
+        <v>256</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>8.09</v>
+        <v>1.52</v>
       </c>
       <c r="I3" t="n">
-        <v>100</v>
+        <v>99.84999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>12.77</v>
+        <v>1.45</v>
       </c>
       <c r="K3" t="n">
-        <v>56.03</v>
+        <v>95.66</v>
       </c>
       <c r="L3" t="n">
-        <v>3.17</v>
+        <v>1.6</v>
       </c>
       <c r="M3" t="n">
-        <v>81.72</v>
+        <v>81.79000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>llama3.1-sft-unbiased-q4_k_m_latest</t>
+          <t>mistralai_ministral-8b-2512</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1100</v>
+        <v>660</v>
       </c>
       <c r="C4" t="n">
-        <v>69</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>179</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
-        <v>353</v>
+        <v>373</v>
       </c>
       <c r="F4" t="n">
-        <v>499</v>
+        <v>269</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>6.27</v>
+        <v>1.37</v>
       </c>
       <c r="I4" t="n">
-        <v>100</v>
+        <v>99.55</v>
       </c>
       <c r="J4" t="n">
-        <v>11.7</v>
+        <v>2.03</v>
       </c>
       <c r="K4" t="n">
-        <v>60.64</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="L4" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.64</v>
       </c>
       <c r="M4" t="n">
-        <v>93.09999999999999</v>
+        <v>86.22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>deepseek_deepseek-v4-flash</t>
+          <t>minimax_minimax-m3</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1100</v>
+        <v>660</v>
       </c>
       <c r="C5" t="n">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>117</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>416</v>
+        <v>324</v>
       </c>
       <c r="F5" t="n">
-        <v>500</v>
+        <v>252</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H5" t="n">
-        <v>6.09</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>100</v>
+        <v>87.88</v>
       </c>
       <c r="J5" t="n">
-        <v>10.64</v>
+        <v>0.64</v>
       </c>
       <c r="K5" t="n">
-        <v>69.5</v>
+        <v>99.36</v>
       </c>
       <c r="L5" t="n">
-        <v>1.31</v>
+        <v>0.74</v>
       </c>
       <c r="M5" t="n">
-        <v>93.28</v>
+        <v>93.68000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>mistral_7b</t>
+          <t>openai_gpt-5.4-mini</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1100</v>
+        <v>660</v>
       </c>
       <c r="C6" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>90</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>560</v>
+        <v>375</v>
       </c>
       <c r="F6" t="n">
-        <v>375</v>
+        <v>280</v>
       </c>
       <c r="G6" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>5.27</v>
+        <v>0.61</v>
       </c>
       <c r="I6" t="n">
-        <v>98.36</v>
+        <v>100</v>
       </c>
       <c r="J6" t="n">
-        <v>7.91</v>
+        <v>0.29</v>
       </c>
       <c r="K6" t="n">
-        <v>80.76000000000001</v>
+        <v>99.70999999999999</v>
       </c>
       <c r="L6" t="n">
-        <v>2.47</v>
+        <v>0.96</v>
       </c>
       <c r="M6" t="n">
-        <v>71.29000000000001</v>
+        <v>89.17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>xiaomi_mimo-v2-flash</t>
+          <t>deepseek_deepseek-v4-flash</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1100</v>
+        <v>660</v>
       </c>
       <c r="C7" t="n">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>76</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>489</v>
+        <v>383</v>
       </c>
       <c r="F7" t="n">
-        <v>486</v>
+        <v>249</v>
       </c>
       <c r="G7" t="n">
+        <v>24</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="I7" t="n">
+        <v>96.36</v>
+      </c>
+      <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="H7" t="n">
-        <v>4.45</v>
-      </c>
-      <c r="I7" t="n">
+      <c r="K7" t="n">
         <v>100</v>
       </c>
-      <c r="J7" t="n">
-        <v>7.62</v>
-      </c>
-      <c r="K7" t="n">
-        <v>80.5</v>
-      </c>
       <c r="L7" t="n">
-        <v>1.12</v>
+        <v>0.98</v>
       </c>
       <c r="M7" t="n">
-        <v>90.67</v>
+        <v>81.11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>x-ai_grok-4.3</t>
+          <t>moonshotai_kimi-k2.6</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1100</v>
+        <v>660</v>
       </c>
       <c r="C8" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>564</v>
+        <v>407</v>
       </c>
       <c r="F8" t="n">
-        <v>478</v>
+        <v>248</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>2.18</v>
+        <v>0.46</v>
       </c>
       <c r="I8" t="n">
-        <v>100</v>
+        <v>99.84999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>3.55</v>
+        <v>0.29</v>
       </c>
       <c r="K8" t="n">
-        <v>90.95999999999999</v>
+        <v>99.42</v>
       </c>
       <c r="L8" t="n">
-        <v>0.75</v>
+        <v>0.64</v>
       </c>
       <c r="M8" t="n">
-        <v>89.18000000000001</v>
+        <v>78.98</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>anthropic_claude-haiku-4.5</t>
+          <t>qwen_qwen3.6-flash</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1100</v>
+        <v>660</v>
       </c>
       <c r="C9" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>633</v>
+        <v>383</v>
       </c>
       <c r="F9" t="n">
-        <v>438</v>
+        <v>267</v>
       </c>
       <c r="G9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="I9" t="n">
+        <v>99.09</v>
+      </c>
+      <c r="J9" t="n">
         <v>0</v>
       </c>
-      <c r="H9" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="I9" t="n">
+      <c r="K9" t="n">
         <v>100</v>
       </c>
-      <c r="J9" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="K9" t="n">
-        <v>95.73999999999999</v>
-      </c>
       <c r="L9" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.96</v>
       </c>
       <c r="M9" t="n">
-        <v>81.72</v>
+        <v>85.58</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>moonshotai_kimi-k2.6</t>
+          <t>x-ai_grok-4.3</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1100</v>
+        <v>660</v>
       </c>
       <c r="C10" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>543</v>
+        <v>450</v>
       </c>
       <c r="F10" t="n">
-        <v>511</v>
+        <v>208</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>1.36</v>
+        <v>0.3</v>
       </c>
       <c r="I10" t="n">
         <v>100</v>
       </c>
       <c r="J10" t="n">
-        <v>1.95</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>92.91</v>
+        <v>100</v>
       </c>
       <c r="L10" t="n">
-        <v>0.75</v>
+        <v>0.64</v>
       </c>
       <c r="M10" t="n">
-        <v>95.34</v>
+        <v>66.23999999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>qwen_qwen3.6-flash</t>
+          <t>google_gemini-3.1-flash-lite</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1100</v>
+        <v>660</v>
       </c>
       <c r="C11" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>550</v>
+        <v>425</v>
       </c>
       <c r="F11" t="n">
-        <v>503</v>
+        <v>233</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>1.09</v>
+        <v>0.15</v>
       </c>
       <c r="I11" t="n">
         <v>100</v>
       </c>
       <c r="J11" t="n">
-        <v>1.42</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>92.91</v>
+        <v>99.70999999999999</v>
       </c>
       <c r="L11" t="n">
-        <v>0.75</v>
+        <v>0.32</v>
       </c>
       <c r="M11" t="n">
-        <v>93.84</v>
+        <v>74.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>google_gemini-3.1-flash-lite</t>
+          <t>anthropic_claude-haiku-4.5</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1100</v>
+        <v>660</v>
       </c>
       <c r="C12" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>601</v>
+        <v>412</v>
       </c>
       <c r="F12" t="n">
-        <v>476</v>
+        <v>248</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
         <v>100</v>
       </c>
       <c r="J12" t="n">
-        <v>1.24</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>96.98999999999999</v>
+        <v>100</v>
       </c>
       <c r="L12" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>88.81</v>
+        <v>78.98</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>minimax_minimax-m2.7</t>
+          <t>xiaomi_mimo-v2-flash</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>11</v>
+        <v>660</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>396</v>
+      </c>
+      <c r="F13" t="n">
+        <v>262</v>
+      </c>
+      <c r="G13" t="n">
         <v>0</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>11</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>83.44</v>
       </c>
     </row>
   </sheetData>
@@ -1363,7 +1363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1405,13 +1405,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>87</v>
+        <v>52</v>
       </c>
       <c r="D2" t="n">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="E2" t="n">
-        <v>73.56</v>
+        <v>82.69</v>
       </c>
     </row>
     <row r="3">
@@ -1426,13 +1426,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D3" t="n">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="E3" t="n">
-        <v>73.33</v>
+        <v>58.54</v>
       </c>
     </row>
     <row r="4">
@@ -1447,13 +1447,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>57</v>
       </c>
       <c r="D4" t="n">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="E4" t="n">
-        <v>78</v>
+        <v>56.14</v>
       </c>
     </row>
     <row r="5">
@@ -1468,13 +1468,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="D5" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E5" t="n">
-        <v>61</v>
+        <v>43.18</v>
       </c>
     </row>
     <row r="6">
@@ -1489,13 +1489,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="D6" t="n">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E6" t="n">
-        <v>74.59999999999999</v>
+        <v>67.34999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -1510,13 +1510,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="D7" t="n">
-        <v>77</v>
+        <v>8</v>
       </c>
       <c r="E7" t="n">
-        <v>77</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -1531,13 +1531,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>100</v>
+        <v>23</v>
       </c>
       <c r="D8" t="n">
-        <v>59</v>
+        <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>59</v>
+        <v>30.43</v>
       </c>
     </row>
     <row r="9">
@@ -1552,13 +1552,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>84</v>
+        <v>37</v>
       </c>
       <c r="D9" t="n">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="E9" t="n">
-        <v>64.29000000000001</v>
+        <v>67.56999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -1573,13 +1573,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>100</v>
+        <v>47</v>
       </c>
       <c r="D10" t="n">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="E10" t="n">
-        <v>72</v>
+        <v>85.11</v>
       </c>
     </row>
     <row r="11">
@@ -1594,13 +1594,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>87</v>
+        <v>60</v>
       </c>
       <c r="D11" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="E11" t="n">
-        <v>54.02</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="12">
@@ -1618,10 +1618,10 @@
         <v>59</v>
       </c>
       <c r="D12" t="n">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="E12" t="n">
-        <v>37.29</v>
+        <v>69.48999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -1636,13 +1636,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="D13" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E13" t="n">
-        <v>29</v>
+        <v>55.93</v>
       </c>
     </row>
     <row r="14">
@@ -1657,13 +1657,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="D14" t="n">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="E14" t="n">
-        <v>37</v>
+        <v>45.76</v>
       </c>
     </row>
     <row r="15">
@@ -1678,13 +1678,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D15" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E15" t="n">
-        <v>61.9</v>
+        <v>71.19</v>
       </c>
     </row>
     <row r="16">
@@ -1699,13 +1699,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D16" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E16" t="n">
-        <v>26</v>
+        <v>53.33</v>
       </c>
     </row>
     <row r="17">
@@ -1720,13 +1720,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>100</v>
+        <v>57</v>
       </c>
       <c r="D17" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="E17" t="n">
-        <v>42</v>
+        <v>43.86</v>
       </c>
     </row>
     <row r="18">
@@ -1741,13 +1741,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="D18" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E18" t="n">
-        <v>38.1</v>
+        <v>64.41</v>
       </c>
     </row>
     <row r="19">
@@ -1762,13 +1762,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D19" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E19" t="n">
-        <v>46</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20">
@@ -1783,13 +1783,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="D20" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="E20" t="n">
-        <v>91.95</v>
+        <v>77.59</v>
       </c>
     </row>
     <row r="21">
@@ -1807,10 +1807,10 @@
         <v>60</v>
       </c>
       <c r="D21" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E21" t="n">
-        <v>75</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="22">
@@ -1825,13 +1825,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="D22" t="n">
-        <v>94</v>
+        <v>34</v>
       </c>
       <c r="E22" t="n">
-        <v>94</v>
+        <v>58.62</v>
       </c>
     </row>
     <row r="23">
@@ -1846,13 +1846,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="D23" t="n">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E23" t="n">
-        <v>79</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -1867,13 +1867,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D24" t="n">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="E24" t="n">
-        <v>92.06</v>
+        <v>69.48999999999999</v>
       </c>
     </row>
     <row r="25">
@@ -1888,13 +1888,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>98</v>
+        <v>45</v>
       </c>
       <c r="D25" t="n">
-        <v>84</v>
+        <v>24</v>
       </c>
       <c r="E25" t="n">
-        <v>85.70999999999999</v>
+        <v>53.33</v>
       </c>
     </row>
     <row r="26">
@@ -1909,13 +1909,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="D26" t="n">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="E26" t="n">
-        <v>86.87</v>
+        <v>55.77</v>
       </c>
     </row>
     <row r="27">
@@ -1930,13 +1930,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="D27" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="E27" t="n">
-        <v>83.33</v>
+        <v>67.8</v>
       </c>
     </row>
     <row r="28">
@@ -1951,13 +1951,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="D28" t="n">
-        <v>92</v>
+        <v>48</v>
       </c>
       <c r="E28" t="n">
-        <v>92</v>
+        <v>81.36</v>
       </c>
     </row>
     <row r="29">
@@ -1972,13 +1972,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>87</v>
+        <v>60</v>
       </c>
       <c r="D29" t="n">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="E29" t="n">
-        <v>63.22</v>
+        <v>56.67</v>
       </c>
     </row>
     <row r="30">
@@ -1996,10 +1996,10 @@
         <v>60</v>
       </c>
       <c r="D30" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="E30" t="n">
-        <v>71.67</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31">
@@ -2014,13 +2014,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="D31" t="n">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="E31" t="n">
-        <v>68</v>
+        <v>57.63</v>
       </c>
     </row>
     <row r="32">
@@ -2035,13 +2035,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D32" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="E32" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33">
@@ -2056,13 +2056,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D33" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E33" t="n">
-        <v>74.59999999999999</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34">
@@ -2077,13 +2077,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D34" t="n">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="E34" t="n">
-        <v>56</v>
+        <v>51.67</v>
       </c>
     </row>
     <row r="35">
@@ -2098,13 +2098,13 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D35" t="n">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="E35" t="n">
-        <v>49</v>
+        <v>46.67</v>
       </c>
     </row>
     <row r="36">
@@ -2119,13 +2119,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="D36" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="E36" t="n">
-        <v>59.52</v>
+        <v>61.67</v>
       </c>
     </row>
     <row r="37">
@@ -2140,13 +2140,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D37" t="n">
-        <v>80</v>
+        <v>42</v>
       </c>
       <c r="E37" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38">
@@ -2161,13 +2161,13 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="D38" t="n">
-        <v>84</v>
+        <v>32</v>
       </c>
       <c r="E38" t="n">
-        <v>96.55</v>
+        <v>58.18</v>
       </c>
     </row>
     <row r="39">
@@ -2182,13 +2182,13 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D39" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="E39" t="n">
-        <v>92.59</v>
+        <v>61.54</v>
       </c>
     </row>
     <row r="40">
@@ -2203,13 +2203,13 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="D40" t="n">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="E40" t="n">
-        <v>96</v>
+        <v>61.82</v>
       </c>
     </row>
     <row r="41">
@@ -2224,13 +2224,13 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>99</v>
+        <v>55</v>
       </c>
       <c r="D41" t="n">
-        <v>90</v>
+        <v>32</v>
       </c>
       <c r="E41" t="n">
-        <v>90.91</v>
+        <v>58.18</v>
       </c>
     </row>
     <row r="42">
@@ -2245,13 +2245,13 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D42" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="E42" t="n">
-        <v>95.23999999999999</v>
+        <v>54.24</v>
       </c>
     </row>
     <row r="43">
@@ -2266,13 +2266,13 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>84</v>
+        <v>40</v>
       </c>
       <c r="D43" t="n">
-        <v>76</v>
+        <v>19</v>
       </c>
       <c r="E43" t="n">
-        <v>90.48</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="44">
@@ -2287,13 +2287,13 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="D44" t="n">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="E44" t="n">
-        <v>92.13</v>
+        <v>45.24</v>
       </c>
     </row>
     <row r="45">
@@ -2308,13 +2308,13 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="D45" t="n">
-        <v>75</v>
+        <v>23</v>
       </c>
       <c r="E45" t="n">
-        <v>94.94</v>
+        <v>56.1</v>
       </c>
     </row>
     <row r="46">
@@ -2329,19 +2329,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>95</v>
+        <v>55</v>
       </c>
       <c r="D46" t="n">
-        <v>92</v>
+        <v>36</v>
       </c>
       <c r="E46" t="n">
-        <v>96.84</v>
+        <v>65.45</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>mistral_7b</t>
+          <t>minimax_minimax-m3</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2350,19 +2350,19 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="D47" t="n">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="E47" t="n">
-        <v>98.84999999999999</v>
+        <v>72.22</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>mistral_7b</t>
+          <t>minimax_minimax-m3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2371,19 +2371,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="D48" t="n">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E48" t="n">
-        <v>100</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>mistral_7b</t>
+          <t>minimax_minimax-m3</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2392,19 +2392,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="D49" t="n">
-        <v>99</v>
+        <v>21</v>
       </c>
       <c r="E49" t="n">
-        <v>99</v>
+        <v>55.26</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>mistral_7b</t>
+          <t>minimax_minimax-m3</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2413,19 +2413,19 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="D50" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="E50" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>mistral_7b</t>
+          <t>minimax_minimax-m3</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2434,19 +2434,19 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="D51" t="n">
-        <v>61</v>
+        <v>28</v>
       </c>
       <c r="E51" t="n">
-        <v>98.39</v>
+        <v>75.68000000000001</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>mistral_7b</t>
+          <t>minimax_minimax-m3</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2455,19 +2455,19 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>88</v>
+        <v>43</v>
       </c>
       <c r="D52" t="n">
-        <v>88</v>
+        <v>21</v>
       </c>
       <c r="E52" t="n">
-        <v>100</v>
+        <v>48.84</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>mistral_7b</t>
+          <t>minimax_minimax-m3</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2476,19 +2476,19 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>88</v>
+        <v>46</v>
       </c>
       <c r="D53" t="n">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="E53" t="n">
-        <v>100</v>
+        <v>36.96</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>mistral_7b</t>
+          <t>minimax_minimax-m3</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2497,19 +2497,19 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="D54" t="n">
-        <v>81</v>
+        <v>28</v>
       </c>
       <c r="E54" t="n">
-        <v>98.78</v>
+        <v>59.57</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>mistral_7b</t>
+          <t>minimax_minimax-m3</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2518,19 +2518,19 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>99</v>
+        <v>40</v>
       </c>
       <c r="D55" t="n">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="E55" t="n">
-        <v>98.98999999999999</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>moonshotai_kimi-k2.6</t>
+          <t>mistralai_ministral-8b-2512</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2539,19 +2539,19 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>87</v>
+        <v>52</v>
       </c>
       <c r="D56" t="n">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="E56" t="n">
-        <v>70.11</v>
+        <v>65.38</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>moonshotai_kimi-k2.6</t>
+          <t>mistralai_ministral-8b-2512</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2560,19 +2560,19 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="D57" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E57" t="n">
-        <v>51.67</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>moonshotai_kimi-k2.6</t>
+          <t>mistralai_ministral-8b-2512</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2581,19 +2581,19 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="D58" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="E58" t="n">
-        <v>61</v>
+        <v>67.34999999999999</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>moonshotai_kimi-k2.6</t>
+          <t>mistralai_ministral-8b-2512</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2602,19 +2602,19 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="D59" t="n">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="E59" t="n">
-        <v>43</v>
+        <v>47.83</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>moonshotai_kimi-k2.6</t>
+          <t>mistralai_ministral-8b-2512</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2623,19 +2623,19 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="D60" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E60" t="n">
-        <v>60.32</v>
+        <v>62</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>moonshotai_kimi-k2.6</t>
+          <t>mistralai_ministral-8b-2512</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2644,19 +2644,19 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="D61" t="n">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="E61" t="n">
-        <v>44</v>
+        <v>45.71</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>moonshotai_kimi-k2.6</t>
+          <t>mistralai_ministral-8b-2512</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2665,19 +2665,19 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="D62" t="n">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="E62" t="n">
-        <v>43</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>moonshotai_kimi-k2.6</t>
+          <t>mistralai_ministral-8b-2512</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2686,19 +2686,19 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>84</v>
+        <v>40</v>
       </c>
       <c r="D63" t="n">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="E63" t="n">
-        <v>46.43</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>moonshotai_kimi-k2.6</t>
+          <t>mistralai_ministral-8b-2512</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2707,19 +2707,19 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D64" t="n">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="E64" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>openai_gpt-5.4-nano</t>
+          <t>moonshotai_kimi-k2.6</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2728,19 +2728,19 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>87</v>
+        <v>60</v>
       </c>
       <c r="D65" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="E65" t="n">
-        <v>26.44</v>
+        <v>76.67</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>openai_gpt-5.4-nano</t>
+          <t>moonshotai_kimi-k2.6</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2749,19 +2749,19 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D66" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E66" t="n">
-        <v>45</v>
+        <v>63.79</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>openai_gpt-5.4-nano</t>
+          <t>moonshotai_kimi-k2.6</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2770,19 +2770,19 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D67" t="n">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="E67" t="n">
-        <v>27</v>
+        <v>65</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>openai_gpt-5.4-nano</t>
+          <t>moonshotai_kimi-k2.6</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2791,19 +2791,19 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D68" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E68" t="n">
-        <v>30</v>
+        <v>38.33</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>openai_gpt-5.4-nano</t>
+          <t>moonshotai_kimi-k2.6</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2812,19 +2812,19 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D69" t="n">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="E69" t="n">
-        <v>38.1</v>
+        <v>71.67</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>openai_gpt-5.4-nano</t>
+          <t>moonshotai_kimi-k2.6</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2833,19 +2833,19 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>100</v>
+        <v>57</v>
       </c>
       <c r="D70" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E70" t="n">
-        <v>33</v>
+        <v>43.86</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>openai_gpt-5.4-nano</t>
+          <t>moonshotai_kimi-k2.6</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2854,19 +2854,19 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="D71" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E71" t="n">
-        <v>38</v>
+        <v>50.91</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>openai_gpt-5.4-nano</t>
+          <t>moonshotai_kimi-k2.6</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2875,19 +2875,19 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>84</v>
+        <v>57</v>
       </c>
       <c r="D72" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E72" t="n">
-        <v>46.43</v>
+        <v>63.16</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>openai_gpt-5.4-nano</t>
+          <t>moonshotai_kimi-k2.6</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2896,19 +2896,19 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="D73" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="E73" t="n">
-        <v>40</v>
+        <v>83.05</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>qwen_qwen3.6-flash</t>
+          <t>openai_gpt-5.4-mini</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2917,19 +2917,19 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>87</v>
+        <v>60</v>
       </c>
       <c r="D74" t="n">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="E74" t="n">
-        <v>87.36</v>
+        <v>68.33</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>qwen_qwen3.6-flash</t>
+          <t>openai_gpt-5.4-mini</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2941,16 +2941,16 @@
         <v>60</v>
       </c>
       <c r="D75" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="E75" t="n">
-        <v>73.33</v>
+        <v>58.33</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>qwen_qwen3.6-flash</t>
+          <t>openai_gpt-5.4-mini</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2959,19 +2959,19 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D76" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E76" t="n">
-        <v>83</v>
+        <v>56.67</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>qwen_qwen3.6-flash</t>
+          <t>openai_gpt-5.4-mini</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2980,19 +2980,19 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D77" t="n">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="E77" t="n">
-        <v>69</v>
+        <v>45</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>qwen_qwen3.6-flash</t>
+          <t>openai_gpt-5.4-mini</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3001,19 +3001,19 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D78" t="n">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="E78" t="n">
-        <v>84.13</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>qwen_qwen3.6-flash</t>
+          <t>openai_gpt-5.4-mini</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3022,19 +3022,19 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D79" t="n">
-        <v>70</v>
+        <v>17</v>
       </c>
       <c r="E79" t="n">
-        <v>70</v>
+        <v>28.33</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>qwen_qwen3.6-flash</t>
+          <t>openai_gpt-5.4-mini</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3043,19 +3043,19 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D80" t="n">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="E80" t="n">
-        <v>78</v>
+        <v>48.33</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>qwen_qwen3.6-flash</t>
+          <t>openai_gpt-5.4-mini</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3064,19 +3064,19 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="D81" t="n">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="E81" t="n">
-        <v>78.56999999999999</v>
+        <v>53.33</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>qwen_qwen3.6-flash</t>
+          <t>openai_gpt-5.4-mini</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3085,19 +3085,19 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D82" t="n">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="E82" t="n">
-        <v>84</v>
+        <v>76.67</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>x-ai_grok-4.3</t>
+          <t>qwen_qwen3.6-flash</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3106,19 +3106,19 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="D83" t="n">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="E83" t="n">
-        <v>95.40000000000001</v>
+        <v>74.14</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>x-ai_grok-4.3</t>
+          <t>qwen_qwen3.6-flash</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3127,19 +3127,19 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D84" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="E84" t="n">
-        <v>76.67</v>
+        <v>68.97</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>x-ai_grok-4.3</t>
+          <t>qwen_qwen3.6-flash</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3148,19 +3148,19 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D85" t="n">
-        <v>87</v>
+        <v>31</v>
       </c>
       <c r="E85" t="n">
-        <v>87</v>
+        <v>51.67</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>x-ai_grok-4.3</t>
+          <t>qwen_qwen3.6-flash</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -3169,19 +3169,19 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="D86" t="n">
-        <v>93</v>
+        <v>29</v>
       </c>
       <c r="E86" t="n">
-        <v>93</v>
+        <v>50</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>x-ai_grok-4.3</t>
+          <t>qwen_qwen3.6-flash</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3190,19 +3190,19 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D87" t="n">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="E87" t="n">
-        <v>93.65000000000001</v>
+        <v>70.18000000000001</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>x-ai_grok-4.3</t>
+          <t>qwen_qwen3.6-flash</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -3211,19 +3211,19 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="D88" t="n">
-        <v>77</v>
+        <v>31</v>
       </c>
       <c r="E88" t="n">
-        <v>77</v>
+        <v>56.36</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>x-ai_grok-4.3</t>
+          <t>qwen_qwen3.6-flash</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3232,19 +3232,19 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="D89" t="n">
-        <v>98</v>
+        <v>35</v>
       </c>
       <c r="E89" t="n">
-        <v>98</v>
+        <v>60.34</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>x-ai_grok-4.3</t>
+          <t>qwen_qwen3.6-flash</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3253,19 +3253,19 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="D90" t="n">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="E90" t="n">
-        <v>91.67</v>
+        <v>75</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>x-ai_grok-4.3</t>
+          <t>qwen_qwen3.6-flash</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -3274,19 +3274,19 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="D91" t="n">
-        <v>85</v>
+        <v>42</v>
       </c>
       <c r="E91" t="n">
-        <v>85</v>
+        <v>72.41</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>xiaomi_mimo-v2-flash</t>
+          <t>x-ai_grok-4.3</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -3295,19 +3295,19 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="D92" t="n">
-        <v>87</v>
+        <v>37</v>
       </c>
       <c r="E92" t="n">
-        <v>100</v>
+        <v>63.79</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>xiaomi_mimo-v2-flash</t>
+          <t>x-ai_grok-4.3</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3316,19 +3316,19 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D93" t="n">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="E93" t="n">
-        <v>100</v>
+        <v>53.45</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>xiaomi_mimo-v2-flash</t>
+          <t>x-ai_grok-4.3</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -3337,19 +3337,19 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="D94" t="n">
-        <v>100</v>
+        <v>29</v>
       </c>
       <c r="E94" t="n">
-        <v>100</v>
+        <v>49.15</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>xiaomi_mimo-v2-flash</t>
+          <t>x-ai_grok-4.3</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -3358,19 +3358,19 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D95" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="E95" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>xiaomi_mimo-v2-flash</t>
+          <t>x-ai_grok-4.3</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3379,19 +3379,19 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D96" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="E96" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>xiaomi_mimo-v2-flash</t>
+          <t>x-ai_grok-4.3</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3400,19 +3400,19 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>100</v>
+        <v>57</v>
       </c>
       <c r="D97" t="n">
-        <v>100</v>
+        <v>29</v>
       </c>
       <c r="E97" t="n">
-        <v>100</v>
+        <v>50.88</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>xiaomi_mimo-v2-flash</t>
+          <t>x-ai_grok-4.3</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3421,19 +3421,19 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D98" t="n">
-        <v>100</v>
+        <v>26</v>
       </c>
       <c r="E98" t="n">
-        <v>100</v>
+        <v>43.33</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>xiaomi_mimo-v2-flash</t>
+          <t>x-ai_grok-4.3</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3442,34 +3442,223 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="D99" t="n">
-        <v>84</v>
+        <v>40</v>
       </c>
       <c r="E99" t="n">
-        <v>100</v>
+        <v>67.8</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
+          <t>x-ai_grok-4.3</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>socioeconomic</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>59</v>
+      </c>
+      <c r="D100" t="n">
+        <v>46</v>
+      </c>
+      <c r="E100" t="n">
+        <v>77.97</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
           <t>xiaomi_mimo-v2-flash</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>58</v>
+      </c>
+      <c r="D101" t="n">
+        <v>35</v>
+      </c>
+      <c r="E101" t="n">
+        <v>60.34</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>xiaomi_mimo-v2-flash</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>disability</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>54</v>
+      </c>
+      <c r="D102" t="n">
+        <v>31</v>
+      </c>
+      <c r="E102" t="n">
+        <v>57.41</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>xiaomi_mimo-v2-flash</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>57</v>
+      </c>
+      <c r="D103" t="n">
+        <v>33</v>
+      </c>
+      <c r="E103" t="n">
+        <v>57.89</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>xiaomi_mimo-v2-flash</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>nationality</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>58</v>
+      </c>
+      <c r="D104" t="n">
+        <v>25</v>
+      </c>
+      <c r="E104" t="n">
+        <v>43.1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>xiaomi_mimo-v2-flash</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>physical-appearance</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>57</v>
+      </c>
+      <c r="D105" t="n">
+        <v>35</v>
+      </c>
+      <c r="E105" t="n">
+        <v>61.4</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>xiaomi_mimo-v2-flash</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>race-color</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>39</v>
+      </c>
+      <c r="D106" t="n">
+        <v>15</v>
+      </c>
+      <c r="E106" t="n">
+        <v>38.46</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>xiaomi_mimo-v2-flash</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>religion</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>46</v>
+      </c>
+      <c r="D107" t="n">
+        <v>17</v>
+      </c>
+      <c r="E107" t="n">
+        <v>36.96</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>xiaomi_mimo-v2-flash</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>sexual-orientation</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>54</v>
+      </c>
+      <c r="D108" t="n">
+        <v>29</v>
+      </c>
+      <c r="E108" t="n">
+        <v>53.7</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>xiaomi_mimo-v2-flash</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
         <is>
           <t>socioeconomic</t>
         </is>
       </c>
-      <c r="C100" t="n">
-        <v>100</v>
-      </c>
-      <c r="D100" t="n">
-        <v>100</v>
-      </c>
-      <c r="E100" t="n">
-        <v>100</v>
+      <c r="C109" t="n">
+        <v>59</v>
+      </c>
+      <c r="D109" t="n">
+        <v>41</v>
+      </c>
+      <c r="E109" t="n">
+        <v>69.48999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>